<commit_message>
Give session 21 a VMTW chair and link; Dr. Bazani Shaik becomes co-chair
Session 21, Industrial IoT, Edge Intelligence and Predictive Maintenance (Tuesday
11:25-12:37), was the last session without a joining link. At the committee's
instruction, K. Naga Maha Lakshmi, a VMTW standby volunteer who is free at that time
(her own paper presents on Monday), now chairs it with the Meet link she supplied.
Dr. Bazani Shaik stays on as co-chair. All 60 sessions now have a link. The session 21
chair sheet is regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/programme/chair-sheets/S21.xlsx
+++ b/programme/chair-sheets/S21.xlsx
@@ -46,19 +46,19 @@
     <t xml:space="preserve">Session chair</t>
   </si>
   <si>
+    <t xml:space="preserve">K. Naga Maha Lakshmi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-chair</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dr. Bazani Shaik</t>
   </si>
   <si>
-    <t xml:space="preserve">Co-chair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Joining link</t>
   </si>
   <si>
-    <t xml:space="preserve">to be confirmed</t>
+    <t xml:space="preserve">https://meet.google.com/jjg-skto-rev</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>

</xml_diff>